<commit_message>
US-28: In ra may in mac dinh, them so thung vao Template_v1
- Station.Wpf: bo LabelPrint:PrinterName, Excel/LibreOffice luon in ra may in mac dinh Windows
- Template_v1: vung QR gop A1:A5, A6 = {{BoxNo}} (dung bo cuc tem PrintLabel cu)
- docs: cap nhat US-28

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Template_v1.xlsx
+++ b/templates/Template_v1.xlsx
@@ -37,6 +37,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
+    <x:t>{{QrCode}}</x:t>
+  </x:si>
+  <x:si>
     <x:t>Code</x:t>
   </x:si>
   <x:si>
@@ -61,16 +64,16 @@
     <x:t>Gross Weight</x:t>
   </x:si>
   <x:si>
+    <x:t>{{GrossWeight}} kg</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Q.C</x:t>
+  </x:si>
+  <x:si>
     <x:t>NV cân: {{OperatorNames}}</x:t>
   </x:si>
   <x:si>
-    <x:t>Q.C</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{QrCode}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{GrossWeight}} kg</x:t>
+    <x:t>{{BoxNo}}</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -130,7 +133,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="7">
+  <x:borders count="10">
     <x:border>
       <x:left/>
       <x:right/>
@@ -216,8 +219,59 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color indexed="64"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color indexed="64"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color indexed="64"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color indexed="64"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color indexed="64"/>
+      </x:right>
+      <x:top style="none">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color indexed="64"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color indexed="64"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color indexed="64"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
   </x:borders>
-  <x:cellStyleXfs count="12">
+  <x:cellStyleXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
@@ -252,8 +306,17 @@
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="7" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="8" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="9" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -337,6 +400,18 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellXfs>
@@ -665,31 +740,31 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:4" ht="79.05" customHeight="1" x14ac:dyDescent="0.3">
-      <x:c r="A1" s="13" t="s">
-        <x:v>10</x:v>
+      <x:c r="A1" s="25" t="s">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="14" t="s">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C1" s="15" t="s">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D1" s="16"/>
     </x:row>
     <x:row r="2" spans="1:4" ht="79.05" customHeight="1" x14ac:dyDescent="0.3">
       <x:c r="A2" s="17"/>
       <x:c r="B2" s="14" t="s">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C2" s="15" t="s">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D2" s="16"/>
     </x:row>
     <x:row r="3" spans="1:4" ht="79.05" customHeight="1" x14ac:dyDescent="0.3">
       <x:c r="A3" s="17"/>
       <x:c r="B3" s="14" t="s">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C3" s="18"/>
       <x:c r="D3" s="19"/>
@@ -697,36 +772,38 @@
     <x:row r="4" spans="1:4" ht="79.05" customHeight="1" x14ac:dyDescent="0.3">
       <x:c r="A4" s="17"/>
       <x:c r="B4" s="14" t="s">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C4" s="15" t="s">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D4" s="16"/>
     </x:row>
     <x:row r="5" spans="1:4" ht="79.05" customHeight="1" x14ac:dyDescent="0.3">
-      <x:c r="A5" s="17"/>
+      <x:c r="A5" s="26"/>
       <x:c r="B5" s="14" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C5" s="20" t="s">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D5" s="21"/>
     </x:row>
     <x:row r="6" spans="1:4" ht="79.05" customHeight="1" x14ac:dyDescent="0.65">
-      <x:c r="A6" s="22"/>
+      <x:c r="A6" s="27" t="s">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="B6" s="14" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C6" s="23"/>
       <x:c r="D6" s="24" t="s">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells count="6">
-    <x:mergeCell ref="A1:A6"/>
+    <x:mergeCell ref="A1:A5"/>
     <x:mergeCell ref="C1:D1"/>
     <x:mergeCell ref="C2:D2"/>
     <x:mergeCell ref="C3:D3"/>

</xml_diff>